<commit_message>
Results for qsvc alone
</commit_message>
<xml_diff>
--- a/compressed_data_classification/src/models/best_models_result/resultados_modelos_original_data.xlsx
+++ b/compressed_data_classification/src/models/best_models_result/resultados_modelos_original_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,121 +471,19 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{'mlp__activation': 'relu', 'mlp__alpha': 0.01, 'mlp__early_stopping': True, 'mlp__hidden_layer_sizes': (20, 10), 'mlp__learning_rate': 'constant', 'mlp__learning_rate_init': 0.001, 'mlp__max_iter': 5000, 'mlp__solver': 'sgd'}</t>
+          <t>{'qsvc__decision_function_shape': 'ovr', 'qsvc__probability': True}</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.0576</v>
+        <v>0.7252999999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5</v>
+        <v>0.9832</v>
       </c>
       <c r="E2" t="n">
-        <v>33.3541</v>
+        <v>19.8941</v>
       </c>
       <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">              precision    recall  f1-score   support
-           0       0.00      0.00      0.00        99
-           1       0.00      0.00      0.00       104
-           2       0.00      0.00      0.00       112
-           3       0.00      0.00      0.00        86
-           4       0.00      0.00      0.00        88
-           5       0.06      1.00      0.11        98
-           6       0.00      0.00      0.00       101
-           7       0.00      0.00      0.00        94
-           8       0.00      0.00      0.00        99
-           9       0.00      0.00      0.00       105
-          10       0.00      0.00      0.00       121
-          11       0.00      0.00      0.00        99
-          12       0.00      0.00      0.00        94
-          13       0.00      0.00      0.00        97
-          14       0.00      0.00      0.00       102
-          15       0.00      0.00      0.00        91
-          16       0.00      0.00      0.00       110
-    accuracy                           0.06      1700
-   macro avg       0.00      0.06      0.01      1700
-weighted avg       0.00      0.06      0.01      1700
-</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>0.059</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.0003</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>{'svc_rbf__C': 1, 'svc_rbf__gamma': 0.01, 'svc_rbf__kernel': 'rbf', 'svc_rbf__probability': True, 'svc_rbf__random_state': 42}</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>0.6624</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.988</v>
-      </c>
-      <c r="E3" t="n">
-        <v>21.62</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">              precision    recall  f1-score   support
-           0       1.00      1.00      1.00        99
-           1       0.95      0.77      0.85       104
-           2       0.99      0.87      0.92       112
-           3       1.00      0.62      0.76        86
-           4       0.94      0.36      0.52        88
-           5       0.97      0.31      0.47        98
-           6       0.99      0.66      0.79       101
-           7       0.91      0.52      0.66        94
-           8       0.86      0.44      0.59        99
-           9       1.00      1.00      1.00       105
-          10       1.00      0.88      0.94       121
-          11       0.96      0.25      0.40        99
-          12       0.53      0.21      0.30        94
-          13       1.00      0.97      0.98        97
-          14       1.00      0.37      0.54       102
-          15       0.14      0.98      0.25        91
-          16       0.94      0.88      0.91       110
-    accuracy                           0.66      1700
-   macro avg       0.89      0.65      0.70      1700
-weighted avg       0.90      0.66      0.71      1700
-</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>0.6415</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.016</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>{'qsvc__probability': True}</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>0.7252999999999999</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.9832</v>
-      </c>
-      <c r="E4" t="n">
-        <v>19.8941</v>
-      </c>
-      <c r="F4" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
            0       0.88      1.00      0.93        99
@@ -611,10 +509,10 @@
 </t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="G2" t="n">
         <v>0.7139</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H2" t="n">
         <v>0.0125</v>
       </c>
     </row>

</xml_diff>

<commit_message>
running just one fold without gridSearch
</commit_message>
<xml_diff>
--- a/compressed_data_classification/src/models/best_models_result/resultados_modelos_original_data.xlsx
+++ b/compressed_data_classification/src/models/best_models_result/resultados_modelos_original_data.xlsx
@@ -425,43 +425,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>melhores_parametros</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
           <t>acuracia</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>roc_auc_score</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>mse</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>relatorio_classificacao</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>best_mean_score</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>std_best_score_k_fold</t>
         </is>
       </c>
     </row>
@@ -469,51 +454,40 @@
       <c r="A2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>{'qsvc__C': 1, 'qsvc__coef0': 1, 'qsvc__decision_function_shape': 'ovo', 'qsvc__degree': 2, 'qsvc__gamma': 'scale', 'qsvc__kernel': 'poly', 'qsvc__probability': True}</t>
-        </is>
+      <c r="B2" t="n">
+        <v>0.9418</v>
       </c>
       <c r="C2" t="n">
-        <v>0.7729</v>
+        <v>0.9976</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9879</v>
-      </c>
-      <c r="E2" t="n">
-        <v>16.0312</v>
-      </c>
-      <c r="F2" t="inlineStr">
+        <v>4.4659</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
-           0       0.89      1.00      0.94        99
-           1       0.52      0.73      0.61       104
-           2       0.86      0.81      0.83       112
-           3       0.78      0.97      0.86        86
-           4       0.79      0.93      0.85        88
-           5       0.87      0.94      0.90        98
-           6       0.84      0.87      0.85       101
-           7       0.78      0.66      0.71        94
-           8       0.67      0.81      0.73        99
-           9       0.97      1.00      0.99       105
-          10       0.66      0.31      0.42       121
-          11       0.94      0.76      0.84        99
-          12       1.00      0.60      0.75        94
-          13       0.85      0.64      0.73        97
-          14       1.00      0.78      0.88       102
-          15       1.00      0.53      0.69        91
-          16       0.46      0.88      0.60       110
-    accuracy                           0.77      1700
-   macro avg       0.81      0.78      0.78      1700
-weighted avg       0.81      0.77      0.77      1700
+           0       0.99      1.00      0.99        99
+           1       0.95      0.84      0.89       104
+           2       0.98      0.99      0.99       112
+           3       1.00      1.00      1.00        86
+           4       0.97      0.99      0.98        88
+           5       0.99      0.99      0.99        98
+           6       0.92      0.94      0.93       101
+           7       0.97      0.79      0.87        94
+           8       0.83      0.92      0.88        99
+           9       0.99      1.00      1.00       105
+          10       0.95      0.93      0.94       121
+          11       0.94      0.93      0.93        99
+          12       0.97      0.88      0.92        94
+          13       0.99      1.00      0.99        97
+          14       1.00      0.96      0.98       102
+          15       0.95      0.92      0.94        91
+          16       0.73      0.93      0.82       110
+    accuracy                           0.94      1700
+   macro avg       0.95      0.94      0.94      1700
+weighted avg       0.95      0.94      0.94      1700
 </t>
         </is>
-      </c>
-      <c r="G2" t="n">
-        <v>0.7607</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.0139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Preparing the algorithm to have max_iter
</commit_message>
<xml_diff>
--- a/compressed_data_classification/src/models/best_models_result/resultados_modelos_original_data.xlsx
+++ b/compressed_data_classification/src/models/best_models_result/resultados_modelos_original_data.xlsx
@@ -455,33 +455,33 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.9418</v>
+        <v>0.9412</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9976</v>
+        <v>0.9977</v>
       </c>
       <c r="D2" t="n">
-        <v>4.4659</v>
+        <v>4.5541</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
-           0       0.99      1.00      0.99        99
-           1       0.95      0.84      0.89       104
-           2       0.98      0.99      0.99       112
+           0       0.98      1.00      0.99        99
+           1       0.96      0.84      0.89       104
+           2       0.97      0.99      0.98       112
            3       1.00      1.00      1.00        86
            4       0.97      0.99      0.98        88
            5       0.99      0.99      0.99        98
            6       0.92      0.94      0.93       101
-           7       0.97      0.79      0.87        94
+           7       0.97      0.78      0.86        94
            8       0.83      0.92      0.88        99
            9       0.99      1.00      1.00       105
           10       0.95      0.93      0.94       121
-          11       0.94      0.93      0.93        99
+          11       0.94      0.94      0.94        99
           12       0.97      0.88      0.92        94
           13       0.99      1.00      0.99        97
           14       1.00      0.96      0.98       102
-          15       0.95      0.92      0.94        91
+          15       0.95      0.91      0.93        91
           16       0.73      0.93      0.82       110
     accuracy                           0.94      1700
    macro avg       0.95      0.94      0.94      1700

</xml_diff>

<commit_message>
Final results - fail
</commit_message>
<xml_diff>
--- a/compressed_data_classification/src/models/best_models_result/resultados_modelos_original_data.xlsx
+++ b/compressed_data_classification/src/models/best_models_result/resultados_modelos_original_data.xlsx
@@ -455,37 +455,37 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>0.9412</v>
+        <v>0.9752999999999999</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9977</v>
+        <v>0.9994</v>
       </c>
       <c r="D2" t="n">
-        <v>4.5541</v>
+        <v>1.6135</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
-           0       0.98      1.00      0.99        99
-           1       0.96      0.84      0.89       104
-           2       0.97      0.99      0.98       112
+           0       1.00      1.00      1.00        99
+           1       0.91      0.97      0.94       104
+           2       0.98      0.99      0.99       112
            3       1.00      1.00      1.00        86
-           4       0.97      0.99      0.98        88
-           5       0.99      0.99      0.99        98
-           6       0.92      0.94      0.93       101
-           7       0.97      0.78      0.86        94
-           8       0.83      0.92      0.88        99
-           9       0.99      1.00      1.00       105
-          10       0.95      0.93      0.94       121
+           4       0.98      0.95      0.97        88
+           5       1.00      1.00      1.00        98
+           6       0.98      0.98      0.98       101
+           7       0.99      0.99      0.99        94
+           8       0.92      0.97      0.95        99
+           9       1.00      1.00      1.00       105
+          10       0.98      0.98      0.98       121
           11       0.94      0.94      0.94        99
-          12       0.97      0.88      0.92        94
+          12       1.00      0.89      0.94        94
           13       0.99      1.00      0.99        97
-          14       1.00      0.96      0.98       102
-          15       0.95      0.91      0.93        91
-          16       0.73      0.93      0.82       110
-    accuracy                           0.94      1700
-   macro avg       0.95      0.94      0.94      1700
-weighted avg       0.95      0.94      0.94      1700
+          14       0.98      0.96      0.97       102
+          15       0.99      0.93      0.96        91
+          16       0.96      1.00      0.98       110
+    accuracy                           0.98      1700
+   macro avg       0.98      0.97      0.98      1700
+weighted avg       0.98      0.98      0.98      1700
 </t>
         </is>
       </c>

</xml_diff>